<commit_message>
Include measured mean latency and derived GPU FPS in 5090 reports
</commit_message>
<xml_diff>
--- a/reports/5090/experiments.xlsx
+++ b/reports/5090/experiments.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Training status" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Query results'!$A$1:$AD$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Query results'!$A$1:$AH$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD25"/>
+  <dimension ref="A1:AH25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,40 +537,60 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>mean_ms</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>median_ms</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>p95_ms</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>fps_from_mean</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>peak_allocated_mib</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>benchmark_status</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>benchmark_reason</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>coverage_05</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>class_correct_coverage_05</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>identity_passed</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
@@ -654,29 +674,41 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
+        <v>7.331793599128723</v>
+      </c>
+      <c r="X2" t="n">
         <v>7.329007863998413</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>7.368627190589905</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
+        <v>136.3922737976197</v>
+      </c>
+      <c r="AA2" t="n">
         <v>212.90283203125</v>
       </c>
-      <c r="Z2" s="2" t="n">
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" s="2" t="n">
         <v>0.7867592043138368</v>
       </c>
-      <c r="AA2" s="2" t="n">
+      <c r="AE2" s="2" t="n">
         <v>0.6538610387264894</v>
       </c>
-      <c r="AB2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG2" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -755,21 +787,31 @@
       <c r="V3" t="n">
         <v>0</v>
       </c>
-      <c r="Z3" s="2" t="n">
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="n">
         <v>0.7600459242250287</v>
       </c>
-      <c r="AA3" s="2" t="n">
+      <c r="AE3" s="2" t="n">
         <v>0.6303099885189437</v>
       </c>
-      <c r="AB3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AF3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -849,29 +891,41 @@
         <v>-0.118657522822814</v>
       </c>
       <c r="W4" t="n">
+        <v>7.298941769599915</v>
+      </c>
+      <c r="X4" t="n">
         <v>7.298352003097534</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>7.327645015716553</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
+        <v>137.0061622035401</v>
+      </c>
+      <c r="AA4" t="n">
         <v>212.90283203125</v>
       </c>
-      <c r="Z4" s="2" t="n">
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" s="2" t="n">
         <v>0.7727753554013261</v>
       </c>
-      <c r="AA4" s="2" t="n">
+      <c r="AE4" s="2" t="n">
         <v>0.6425346371165407</v>
       </c>
-      <c r="AB4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AF4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG4" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -950,21 +1004,31 @@
       <c r="V5" t="n">
         <v>-0.2260136606720239</v>
       </c>
-      <c r="Z5" s="2" t="n">
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD5" s="2" t="n">
         <v>0.7474167623421355</v>
       </c>
-      <c r="AA5" s="2" t="n">
+      <c r="AE5" s="2" t="n">
         <v>0.618828932261768</v>
       </c>
-      <c r="AB5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AF5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1044,29 +1108,41 @@
         <v>-0.3043582651745674</v>
       </c>
       <c r="W6" t="n">
+        <v>7.293236801624298</v>
+      </c>
+      <c r="X6" t="n">
         <v>7.289936065673828</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>7.328998351097107</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
+        <v>137.1133321459255</v>
+      </c>
+      <c r="AA6" t="n">
         <v>212.90283203125</v>
       </c>
-      <c r="Z6" s="2" t="n">
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" s="2" t="n">
         <v>0.7497871462112026</v>
       </c>
-      <c r="AA6" s="2" t="n">
+      <c r="AE6" s="2" t="n">
         <v>0.6243195128873293</v>
       </c>
-      <c r="AB6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AF6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG6" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1145,21 +1221,31 @@
       <c r="V7" t="n">
         <v>-0.4483454731230144</v>
       </c>
-      <c r="Z7" s="2" t="n">
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD7" s="2" t="n">
         <v>0.7106773823191733</v>
       </c>
-      <c r="AA7" s="2" t="n">
+      <c r="AE7" s="2" t="n">
         <v>0.5866819747416763</v>
       </c>
-      <c r="AB7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AF7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1239,29 +1325,41 @@
         <v>-0.6365236057599131</v>
       </c>
       <c r="W8" t="n">
+        <v>7.310774393081665</v>
+      </c>
+      <c r="X8" t="n">
         <v>7.308319807052612</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>7.336531138420105</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
+        <v>136.7844151977006</v>
+      </c>
+      <c r="AA8" t="n">
         <v>212.90283203125</v>
       </c>
-      <c r="Z8" s="2" t="n">
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" s="2" t="n">
         <v>0.7147759230114296</v>
       </c>
-      <c r="AA8" s="2" t="n">
+      <c r="AE8" s="2" t="n">
         <v>0.5959390077143373</v>
       </c>
-      <c r="AB8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AF8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG8" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1340,21 +1438,31 @@
       <c r="V9" t="n">
         <v>-0.7791337925166175</v>
       </c>
-      <c r="Z9" s="2" t="n">
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD9" s="2" t="n">
         <v>0.669345579793341</v>
       </c>
-      <c r="AA9" s="2" t="n">
+      <c r="AE9" s="2" t="n">
         <v>0.5591274397244547</v>
       </c>
-      <c r="AB9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AF9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1433,21 +1541,31 @@
       <c r="V10" t="n">
         <v>0</v>
       </c>
-      <c r="Z10" s="2" t="n">
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD10" s="2" t="n">
         <v>0.002296211251435132</v>
       </c>
-      <c r="AA10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AE10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG10" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1526,21 +1644,31 @@
       <c r="V11" t="n">
         <v>0</v>
       </c>
-      <c r="Z11" s="2" t="n">
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD11" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AA11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AE11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1619,21 +1747,31 @@
       <c r="V12" t="n">
         <v>0</v>
       </c>
-      <c r="Z12" s="2" t="n">
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD12" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AA12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB12" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AE12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG12" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1712,21 +1850,31 @@
       <c r="V13" t="n">
         <v>0</v>
       </c>
-      <c r="Z13" s="2" t="n">
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD13" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AA13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB13" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AE13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG13" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1806,29 +1954,41 @@
         <v>0</v>
       </c>
       <c r="W14" t="n">
+        <v>7.362735362052917</v>
+      </c>
+      <c r="X14" t="n">
         <v>7.362879991531372</v>
       </c>
-      <c r="X14" t="n">
+      <c r="Y14" t="n">
         <v>7.388091158866883</v>
       </c>
-      <c r="Y14" t="n">
+      <c r="Z14" t="n">
+        <v>135.8190877202973</v>
+      </c>
+      <c r="AA14" t="n">
         <v>219.30712890625</v>
       </c>
-      <c r="Z14" s="2" t="n">
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" s="2" t="n">
         <v>0.7912484842230192</v>
       </c>
-      <c r="AA14" s="2" t="n">
+      <c r="AE14" s="2" t="n">
         <v>0.6597693438943213</v>
       </c>
-      <c r="AB14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AF14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG14" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1907,21 +2067,31 @@
       <c r="V15" t="n">
         <v>0</v>
       </c>
-      <c r="Z15" s="2" t="n">
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD15" s="2" t="n">
         <v>0.78300803673938</v>
       </c>
-      <c r="AA15" s="2" t="n">
+      <c r="AE15" s="2" t="n">
         <v>0.6521239954075775</v>
       </c>
-      <c r="AB15" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC15" t="inlineStr">
+      <c r="AF15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG15" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2001,29 +2171,41 @@
         <v>-0.107322217698283</v>
       </c>
       <c r="W16" t="n">
+        <v>7.342940323352813</v>
+      </c>
+      <c r="X16" t="n">
         <v>7.341600179672241</v>
       </c>
-      <c r="X16" t="n">
+      <c r="Y16" t="n">
         <v>7.367910265922546</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Z16" t="n">
+        <v>136.1852277104434</v>
+      </c>
+      <c r="AA16" t="n">
         <v>219.30712890625</v>
       </c>
-      <c r="Z16" s="2" t="n">
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" s="2" t="n">
         <v>0.7762068164813334</v>
       </c>
-      <c r="AA16" s="2" t="n">
+      <c r="AE16" s="2" t="n">
         <v>0.6476947289661756</v>
       </c>
-      <c r="AB16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AF16" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG16" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2102,21 +2284,31 @@
       <c r="V17" t="n">
         <v>-0.2224468318102246</v>
       </c>
-      <c r="Z17" s="2" t="n">
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD17" s="2" t="n">
         <v>0.7611940298507462</v>
       </c>
-      <c r="AA17" s="2" t="n">
+      <c r="AE17" s="2" t="n">
         <v>0.6291618828932262</v>
       </c>
-      <c r="AB17" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AF17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2196,29 +2388,41 @@
         <v>-0.3730212068272273</v>
       </c>
       <c r="W18" t="n">
+        <v>7.326717119216919</v>
+      </c>
+      <c r="X18" t="n">
         <v>7.324479818344116</v>
       </c>
-      <c r="X18" t="n">
+      <c r="Y18" t="n">
         <v>7.356246495246888</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Z18" t="n">
+        <v>136.4867762366783</v>
+      </c>
+      <c r="AA18" t="n">
         <v>219.30712890625</v>
       </c>
-      <c r="Z18" s="2" t="n">
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" s="2" t="n">
         <v>0.7542506256611368</v>
       </c>
-      <c r="AA18" s="2" t="n">
+      <c r="AE18" s="2" t="n">
         <v>0.6303310198921541</v>
       </c>
-      <c r="AB18" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC18" t="inlineStr">
+      <c r="AF18" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG18" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2297,21 +2501,31 @@
       <c r="V19" t="n">
         <v>-0.4583202124489344</v>
       </c>
-      <c r="Z19" s="2" t="n">
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD19" s="2" t="n">
         <v>0.7290470723306545</v>
       </c>
-      <c r="AA19" s="2" t="n">
+      <c r="AE19" s="2" t="n">
         <v>0.6073478760045924</v>
       </c>
-      <c r="AB19" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AF19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG19" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2391,29 +2605,41 @@
         <v>-0.7669162614846057</v>
       </c>
       <c r="W20" t="n">
+        <v>7.3457217502594</v>
+      </c>
+      <c r="X20" t="n">
         <v>7.342911958694458</v>
       </c>
-      <c r="X20" t="n">
+      <c r="Y20" t="n">
         <v>7.37548942565918</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="Z20" t="n">
+        <v>136.1336617419094</v>
+      </c>
+      <c r="AA20" t="n">
         <v>219.30712890625</v>
       </c>
-      <c r="Z20" s="2" t="n">
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" s="2" t="n">
         <v>0.7184653886839186</v>
       </c>
-      <c r="AA20" s="2" t="n">
+      <c r="AE20" s="2" t="n">
         <v>0.6018473128821693</v>
       </c>
-      <c r="AB20" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC20" t="inlineStr">
+      <c r="AF20" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG20" t="inlineStr">
         <is>
           <t>full_val</t>
         </is>
       </c>
-      <c r="AD20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2492,21 +2718,31 @@
       <c r="V21" t="n">
         <v>-0.898788326407382</v>
       </c>
-      <c r="Z21" s="2" t="n">
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD21" s="2" t="n">
         <v>0.6785304247990815</v>
       </c>
-      <c r="AA21" s="2" t="n">
+      <c r="AE21" s="2" t="n">
         <v>0.5694603903559128</v>
       </c>
-      <c r="AB21" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC21" t="inlineStr">
+      <c r="AF21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG21" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2585,21 +2821,31 @@
       <c r="V22" t="n">
         <v>0</v>
       </c>
-      <c r="Z22" s="2" t="n">
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD22" s="2" t="n">
         <v>0.003444316877152698</v>
       </c>
-      <c r="AA22" s="2" t="n">
+      <c r="AE22" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AB22" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC22" t="inlineStr">
+      <c r="AF22" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG22" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2678,21 +2924,31 @@
       <c r="V23" t="n">
         <v>0</v>
       </c>
-      <c r="Z23" s="2" t="n">
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD23" s="2" t="n">
         <v>0.003444316877152698</v>
       </c>
-      <c r="AA23" s="2" t="n">
+      <c r="AE23" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AB23" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC23" t="inlineStr">
+      <c r="AF23" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG23" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2771,21 +3027,31 @@
       <c r="V24" t="n">
         <v>0</v>
       </c>
-      <c r="Z24" s="2" t="n">
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD24" s="2" t="n">
         <v>0.003444316877152698</v>
       </c>
-      <c r="AA24" s="2" t="n">
+      <c r="AE24" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AB24" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC24" t="inlineStr">
+      <c r="AF24" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG24" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2864,24 +3130,34 @@
       <c r="V25" t="n">
         <v>0</v>
       </c>
-      <c r="Z25" s="2" t="n">
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>not_measured</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>未保存计时结果</t>
+        </is>
+      </c>
+      <c r="AD25" s="2" t="n">
         <v>0.003444316877152698</v>
       </c>
-      <c r="AA25" s="2" t="n">
+      <c r="AE25" s="2" t="n">
         <v>0.001148105625717566</v>
       </c>
-      <c r="AB25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC25" t="inlineStr">
+      <c r="AF25" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG25" t="inlineStr">
         <is>
           <t>subset_engineering_check</t>
         </is>
       </c>
-      <c r="AD25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD25"/>
+  <autoFilter ref="A1:AH25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Archive 5090 stage latency attribution in automatic experiment reports
</commit_message>
<xml_diff>
--- a/reports/5090/experiments.xlsx
+++ b/reports/5090/experiments.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet name="Query results" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Training status" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Stage latency" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Query results'!$A$1:$AH$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stage latency'!$A$1:$L$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3366,4 +3368,1401 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>queries</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>mean_ms</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fraction_of_staged_forward</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>round_mean_min_ms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>round_mean_max_ms</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>samples</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>bare_whole_ms</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>staged_whole_ms</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>instrumentation_overhead_percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>backbone_0_to_4</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2.918717186927795</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.3961563457554934</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.917560319900513</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2.920791683197022</v>
+      </c>
+      <c r="I2" t="n">
+        <v>250</v>
+      </c>
+      <c r="J2" t="n">
+        <v>7.328705795288086</v>
+      </c>
+      <c r="K2" t="n">
+        <v>7.367589130401611</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.5305620964962676</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>300</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>neck_encoder_5_to_23</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2.554138751983642</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.3466722569319518</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.550784010887146</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2.560000009536743</v>
+      </c>
+      <c r="I3" t="n">
+        <v>250</v>
+      </c>
+      <c r="J3" t="n">
+        <v>7.328705795288086</v>
+      </c>
+      <c r="K3" t="n">
+        <v>7.367589130401611</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.5305620964962676</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>300</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>input_projection_and_query_selection</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3632144646644592</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.04929895766929938</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.3626553589105606</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.3637984013557434</v>
+      </c>
+      <c r="I4" t="n">
+        <v>250</v>
+      </c>
+      <c r="J4" t="n">
+        <v>7.328705795288086</v>
+      </c>
+      <c r="K4" t="n">
+        <v>7.367589130401611</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.5305620964962676</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>300</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>decoder_and_prediction_heads</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1.501266816139221</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.2037663596011883</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.497284483909607</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.503832955360413</v>
+      </c>
+      <c r="I5" t="n">
+        <v>250</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7.328705795288086</v>
+      </c>
+      <c r="K5" t="n">
+        <v>7.367589130401611</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.5305620964962676</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>300</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>output_assembly</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.03025190400332212</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.004106079134962983</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.02977344006299973</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.03153728000819683</v>
+      </c>
+      <c r="I6" t="n">
+        <v>250</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7.328705795288086</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7.367589130401611</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.5305620964962676</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>backbone_0_to_4</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2.917944323539734</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.3970673541997202</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.917126402854919</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2.918695678710938</v>
+      </c>
+      <c r="I7" t="n">
+        <v>250</v>
+      </c>
+      <c r="J7" t="n">
+        <v>7.313524225234985</v>
+      </c>
+      <c r="K7" t="n">
+        <v>7.348738929748535</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.4815011672764102</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>200</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>neck_encoder_5_to_23</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2.554781701087951</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.3476489946793324</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.550517768859863</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2.558648324012756</v>
+      </c>
+      <c r="I8" t="n">
+        <v>250</v>
+      </c>
+      <c r="J8" t="n">
+        <v>7.313524225234985</v>
+      </c>
+      <c r="K8" t="n">
+        <v>7.348738929748535</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.4815011672764102</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>200</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>input_projection_and_query_selection</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3586082553863525</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.04879861141000198</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.3579865580797195</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.3592339181900024</v>
+      </c>
+      <c r="I9" t="n">
+        <v>250</v>
+      </c>
+      <c r="J9" t="n">
+        <v>7.313524225234985</v>
+      </c>
+      <c r="K9" t="n">
+        <v>7.348738929748535</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.4815011672764102</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>200</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>decoder_and_prediction_heads</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1.487357312202454</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.2023962650491585</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.480534398555756</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.490564482212067</v>
+      </c>
+      <c r="I10" t="n">
+        <v>250</v>
+      </c>
+      <c r="J10" t="n">
+        <v>7.313524225234985</v>
+      </c>
+      <c r="K10" t="n">
+        <v>7.348738929748535</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.4815011672764102</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>200</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>output_assembly</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0300473600178957</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.004088777721611602</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.02964415997266769</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.0303744001686573</v>
+      </c>
+      <c r="I11" t="n">
+        <v>250</v>
+      </c>
+      <c r="J11" t="n">
+        <v>7.313524225234985</v>
+      </c>
+      <c r="K11" t="n">
+        <v>7.348738929748535</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.4815011672764102</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>150</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>backbone_0_to_4</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2.917786489486694</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.3970059618344874</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.917167983055115</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2.918451838493347</v>
+      </c>
+      <c r="I12" t="n">
+        <v>250</v>
+      </c>
+      <c r="J12" t="n">
+        <v>7.319018753051758</v>
+      </c>
+      <c r="K12" t="n">
+        <v>7.349477766036987</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.41616252141079</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>150</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>neck_encoder_5_to_23</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2.552733699798584</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.3473353864127789</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.549329924583435</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2.554019827842712</v>
+      </c>
+      <c r="I13" t="n">
+        <v>250</v>
+      </c>
+      <c r="J13" t="n">
+        <v>7.319018753051758</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7.349477766036987</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.41616252141079</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>150</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>input_projection_and_query_selection</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.3598876163959503</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.04896778082097801</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.3592979216575622</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.3603743994235992</v>
+      </c>
+      <c r="I14" t="n">
+        <v>250</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7.319018753051758</v>
+      </c>
+      <c r="K14" t="n">
+        <v>7.349477766036987</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.41616252141079</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>150</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>decoder_and_prediction_heads</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1.488897281646729</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.2025854528776372</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.484351363182068</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.494609282016754</v>
+      </c>
+      <c r="I15" t="n">
+        <v>250</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7.319018753051758</v>
+      </c>
+      <c r="K15" t="n">
+        <v>7.349477766036987</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.41616252141079</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c0-150e-s0</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>150</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>output_assembly</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.03017267201095819</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0.004105417142751357</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.02984128002077341</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.03061119999736547</v>
+      </c>
+      <c r="I16" t="n">
+        <v>250</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7.319018753051758</v>
+      </c>
+      <c r="K16" t="n">
+        <v>7.349477766036987</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.41616252141079</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>300</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>backbone_0_to_4</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2.921381122589112</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.3931170888243577</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.919795851707458</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2.923324794769287</v>
+      </c>
+      <c r="I17" t="n">
+        <v>250</v>
+      </c>
+      <c r="J17" t="n">
+        <v>7.394399616241455</v>
+      </c>
+      <c r="K17" t="n">
+        <v>7.431325693130493</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.4993789733507503</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>neck_encoder_5_to_23</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2.60891853427887</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0.3510704068172588</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.605567998886108</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.61228542804718</v>
+      </c>
+      <c r="I18" t="n">
+        <v>250</v>
+      </c>
+      <c r="J18" t="n">
+        <v>7.394399616241455</v>
+      </c>
+      <c r="K18" t="n">
+        <v>7.431325693130493</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.4993789733507503</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>300</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>input_projection_and_query_selection</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.3588317440748215</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.04828637027798755</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.358056321144104</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.3597600001096726</v>
+      </c>
+      <c r="I19" t="n">
+        <v>250</v>
+      </c>
+      <c r="J19" t="n">
+        <v>7.394399616241455</v>
+      </c>
+      <c r="K19" t="n">
+        <v>7.431325693130493</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.4993789733507503</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>300</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>decoder_and_prediction_heads</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1.510645886898041</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>0.2032808073927482</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.503959679603577</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.522611198425293</v>
+      </c>
+      <c r="I20" t="n">
+        <v>250</v>
+      </c>
+      <c r="J20" t="n">
+        <v>7.394399616241455</v>
+      </c>
+      <c r="K20" t="n">
+        <v>7.431325693130493</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.4993789733507503</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>300</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>output_assembly</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.03154841603338718</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.004245328133384128</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.03109184004366398</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.03188735995441675</v>
+      </c>
+      <c r="I21" t="n">
+        <v>250</v>
+      </c>
+      <c r="J21" t="n">
+        <v>7.394399616241455</v>
+      </c>
+      <c r="K21" t="n">
+        <v>7.431325693130493</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.4993789733507503</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>200</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>backbone_0_to_4</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2.920699264526367</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0.3936941783137034</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2.919552621841431</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2.921941766738891</v>
+      </c>
+      <c r="I22" t="n">
+        <v>250</v>
+      </c>
+      <c r="J22" t="n">
+        <v>7.389371778488159</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7.41870067024231</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.3969064303887437</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>200</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>neck_encoder_5_to_23</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2.609033235549927</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.3516833137661437</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2.606387224197388</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2.611630101203918</v>
+      </c>
+      <c r="I23" t="n">
+        <v>250</v>
+      </c>
+      <c r="J23" t="n">
+        <v>7.389371778488159</v>
+      </c>
+      <c r="K23" t="n">
+        <v>7.41870067024231</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.3969064303887437</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>200</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>input_projection_and_query_selection</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.3607851516008377</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0.04863185180769043</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.3598822402954102</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.3628364795446396</v>
+      </c>
+      <c r="I24" t="n">
+        <v>250</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7.389371778488159</v>
+      </c>
+      <c r="K24" t="n">
+        <v>7.41870067024231</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.3969064303887437</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>200</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>decoder_and_prediction_heads</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1.497092096328735</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0.2017997709941082</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1.491112961769104</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.501523203849793</v>
+      </c>
+      <c r="I25" t="n">
+        <v>250</v>
+      </c>
+      <c r="J25" t="n">
+        <v>7.389371778488159</v>
+      </c>
+      <c r="K25" t="n">
+        <v>7.41870067024231</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.3969064303887437</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>200</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>output_assembly</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.03109094393998384</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0.004190888043872021</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.03089855995029211</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.03133759986609221</v>
+      </c>
+      <c r="I26" t="n">
+        <v>250</v>
+      </c>
+      <c r="J26" t="n">
+        <v>7.389371778488159</v>
+      </c>
+      <c r="K26" t="n">
+        <v>7.41870067024231</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.3969064303887437</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>150</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>backbone_0_to_4</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2.92083686542511</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0.393335925735443</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.919475202560425</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2.922774405479431</v>
+      </c>
+      <c r="I27" t="n">
+        <v>250</v>
+      </c>
+      <c r="J27" t="n">
+        <v>7.387386743545532</v>
+      </c>
+      <c r="K27" t="n">
+        <v>7.425807495117187</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.520085828797634</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>150</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>neck_encoder_5_to_23</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2.608963589668274</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0.3513373584467128</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2.606817288398743</v>
+      </c>
+      <c r="H28" t="n">
+        <v>2.613002238273621</v>
+      </c>
+      <c r="I28" t="n">
+        <v>250</v>
+      </c>
+      <c r="J28" t="n">
+        <v>7.387386743545532</v>
+      </c>
+      <c r="K28" t="n">
+        <v>7.425807495117187</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.520085828797634</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>150</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>input_projection_and_query_selection</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.3568563197851181</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0.04805623092434967</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.3562918388843536</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.3573023998737335</v>
+      </c>
+      <c r="I29" t="n">
+        <v>250</v>
+      </c>
+      <c r="J29" t="n">
+        <v>7.387386743545532</v>
+      </c>
+      <c r="K29" t="n">
+        <v>7.425807495117187</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.520085828797634</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>150</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>decoder_and_prediction_heads</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1.507577731609344</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0.2030186929301152</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1.497944965362549</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.513211529254913</v>
+      </c>
+      <c r="I30" t="n">
+        <v>250</v>
+      </c>
+      <c r="J30" t="n">
+        <v>7.387386743545532</v>
+      </c>
+      <c r="K30" t="n">
+        <v>7.425807495117187</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.520085828797634</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>5090-c0c2-baselines-20261024-s0-r1/5090-rtdetr-r18-c2-150e-s0</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>150</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>output_assembly</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.03157299203425646</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0.004251792421903903</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.03126080010086298</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.03197887998074293</v>
+      </c>
+      <c r="I31" t="n">
+        <v>250</v>
+      </c>
+      <c r="J31" t="n">
+        <v>7.387386743545532</v>
+      </c>
+      <c r="K31" t="n">
+        <v>7.425807495117187</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.520085828797634</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L31"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>